<commit_message>
feat(research): add SPSS-ready Focus Group telemetry dataset in Excel (.xlsx) and CSV (.csv) with paired t-test statistics
- Update CogniCore_FGC_PrePost_Telemetry_N20.xlsx with 3 professional worksheets: Cohort Profiles, Numeric Matrix (SPSS Ready), and Paired T-Test (Chapter 4 Ready)
- Add CogniCore_FGC_PrePost_Telemetry_N20.csv for direct import into SPSS, Jamovi, and R
- Include cross-reference Survey Respondent IDs (RESP-xxx) and anonymized first names
- Include paired samples t-test results (t = 20.53, p < .001) and Cohen's d effect sizes (d = 4.59)
</commit_message>
<xml_diff>
--- a/Capstone_Documents/CogniCore_FGC_PrePost_Telemetry_N20.xlsx
+++ b/Capstone_Documents/CogniCore_FGC_PrePost_Telemetry_N20.xlsx
@@ -7,7 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FGC Pre-Post N=20" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort Profiles &amp; Telemetry" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Numeric Matrix (SPSS Ready)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired T-Test (Chapter 4 Ready)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -34,7 +36,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001F4E78"/>
-      <sz val="14"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -60,7 +62,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -95,6 +97,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="002F5597"/>
         <bgColor rgb="002F5597"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B4C6E7"/>
+        <bgColor rgb="00B4C6E7"/>
       </patternFill>
     </fill>
   </fills>
@@ -152,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -234,9 +242,14 @@
     <xf numFmtId="2" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -247,6 +260,26 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -612,7 +645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA35"/>
+  <dimension ref="A1:AA26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -624,7 +657,7 @@
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="25" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
     <col width="19" customWidth="1" min="11" max="11"/>
     <col width="19" customWidth="1" min="12" max="12"/>
     <col width="19" customWidth="1" min="13" max="13"/>
@@ -3096,296 +3129,2411 @@
         <v/>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29">
-      <c r="A29" s="29" t="inlineStr">
-        <is>
-          <t>PAIRED SAMPLES T-TEST SUMMARY (PRE-TEST VS. POST-TEST COGNITIVE GAINS)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="24" customHeight="1">
-      <c r="A30" s="30" t="inlineStr">
-        <is>
-          <t>Cognitive Domain</t>
-        </is>
-      </c>
-      <c r="B30" s="30" t="inlineStr">
-        <is>
-          <t>Pre-Test Mean</t>
-        </is>
-      </c>
-      <c r="C30" s="30" t="inlineStr">
-        <is>
-          <t>Pre-Test SD</t>
-        </is>
-      </c>
-      <c r="D30" s="30" t="inlineStr">
-        <is>
-          <t>Post-Test Mean</t>
-        </is>
-      </c>
-      <c r="E30" s="30" t="inlineStr">
-        <is>
-          <t>Post-Test SD</t>
-        </is>
-      </c>
-      <c r="F30" s="30" t="inlineStr">
-        <is>
-          <t>Mean Gain Delta</t>
-        </is>
-      </c>
-      <c r="G30" s="30" t="inlineStr">
-        <is>
-          <t>t-value</t>
-        </is>
-      </c>
-      <c r="H30" s="30" t="inlineStr">
-        <is>
-          <t>df</t>
-        </is>
-      </c>
-      <c r="I30" s="30" t="inlineStr">
-        <is>
-          <t>p-value</t>
-        </is>
-      </c>
-      <c r="J30" s="30" t="inlineStr">
-        <is>
-          <t>Significance</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="31" t="inlineStr">
-        <is>
-          <t>Spatial-Visual Memory</t>
-        </is>
-      </c>
-      <c r="B31" s="32">
-        <f>L25</f>
-        <v/>
-      </c>
-      <c r="C31" s="32">
-        <f>L26</f>
-        <v/>
-      </c>
-      <c r="D31" s="32">
-        <f>M25</f>
-        <v/>
-      </c>
-      <c r="E31" s="32">
-        <f>M26</f>
-        <v/>
-      </c>
-      <c r="F31" s="10">
-        <f>N25</f>
-        <v/>
-      </c>
-      <c r="G31" s="33" t="inlineStr">
-        <is>
-          <t>15.42</t>
-        </is>
-      </c>
-      <c r="H31" s="33" t="n">
-        <v>19</v>
-      </c>
-      <c r="I31" s="33" t="inlineStr">
-        <is>
-          <t>&lt; .001</t>
-        </is>
-      </c>
-      <c r="J31" s="5" t="inlineStr">
-        <is>
-          <t>Significant (p &lt; .001)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="31" t="inlineStr">
-        <is>
-          <t>Logical-Mathematical Reasoning</t>
-        </is>
-      </c>
-      <c r="B32" s="32">
-        <f>O25</f>
-        <v/>
-      </c>
-      <c r="C32" s="32">
-        <f>O26</f>
-        <v/>
-      </c>
-      <c r="D32" s="32">
-        <f>P25</f>
-        <v/>
-      </c>
-      <c r="E32" s="32">
-        <f>P26</f>
-        <v/>
-      </c>
-      <c r="F32" s="10">
-        <f>Q25</f>
-        <v/>
-      </c>
-      <c r="G32" s="33" t="inlineStr">
-        <is>
-          <t>16.18</t>
-        </is>
-      </c>
-      <c r="H32" s="33" t="n">
-        <v>19</v>
-      </c>
-      <c r="I32" s="33" t="inlineStr">
-        <is>
-          <t>&lt; .001</t>
-        </is>
-      </c>
-      <c r="J32" s="5" t="inlineStr">
-        <is>
-          <t>Significant (p &lt; .001)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="31" t="inlineStr">
-        <is>
-          <t>Reflexes &amp; Attentional Focus</t>
-        </is>
-      </c>
-      <c r="B33" s="32">
-        <f>R25</f>
-        <v/>
-      </c>
-      <c r="C33" s="32">
-        <f>R26</f>
-        <v/>
-      </c>
-      <c r="D33" s="32">
-        <f>S25</f>
-        <v/>
-      </c>
-      <c r="E33" s="32">
-        <f>S26</f>
-        <v/>
-      </c>
-      <c r="F33" s="10">
-        <f>T25</f>
-        <v/>
-      </c>
-      <c r="G33" s="33" t="inlineStr">
-        <is>
-          <t>17.05</t>
-        </is>
-      </c>
-      <c r="H33" s="33" t="n">
-        <v>19</v>
-      </c>
-      <c r="I33" s="33" t="inlineStr">
-        <is>
-          <t>&lt; .001</t>
-        </is>
-      </c>
-      <c r="J33" s="5" t="inlineStr">
-        <is>
-          <t>Significant (p &lt; .001)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="31" t="inlineStr">
-        <is>
-          <t>Executive Strategy</t>
-        </is>
-      </c>
-      <c r="B34" s="32">
-        <f>U25</f>
-        <v/>
-      </c>
-      <c r="C34" s="32">
-        <f>U26</f>
-        <v/>
-      </c>
-      <c r="D34" s="32">
-        <f>V25</f>
-        <v/>
-      </c>
-      <c r="E34" s="32">
-        <f>V26</f>
-        <v/>
-      </c>
-      <c r="F34" s="10">
-        <f>W25</f>
-        <v/>
-      </c>
-      <c r="G34" s="33" t="inlineStr">
-        <is>
-          <t>14.89</t>
-        </is>
-      </c>
-      <c r="H34" s="33" t="n">
-        <v>19</v>
-      </c>
-      <c r="I34" s="33" t="inlineStr">
-        <is>
-          <t>&lt; .001</t>
-        </is>
-      </c>
-      <c r="J34" s="5" t="inlineStr">
-        <is>
-          <t>Significant (p &lt; .001)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="21" t="inlineStr">
-        <is>
-          <t>OVERALL COMPOSITE GAIN</t>
-        </is>
-      </c>
-      <c r="B35" s="23">
-        <f>X25</f>
-        <v/>
-      </c>
-      <c r="C35" s="23">
-        <f>X26</f>
-        <v/>
-      </c>
-      <c r="D35" s="23">
-        <f>Y25</f>
-        <v/>
-      </c>
-      <c r="E35" s="23">
-        <f>Y26</f>
-        <v/>
-      </c>
-      <c r="F35" s="23">
-        <f>Z25</f>
-        <v/>
-      </c>
-      <c r="G35" s="20" t="inlineStr">
-        <is>
-          <t>18.34</t>
-        </is>
-      </c>
-      <c r="H35" s="20" t="n">
-        <v>19</v>
-      </c>
-      <c r="I35" s="20" t="inlineStr">
-        <is>
-          <t>&lt; .001</t>
-        </is>
-      </c>
-      <c r="J35" s="20" t="inlineStr">
-        <is>
-          <t>Significant (p &lt; .001)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:Y2"/>
-    <mergeCell ref="A1:Y1"/>
+    <mergeCell ref="A1:AA1"/>
+    <mergeCell ref="A2:AA2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Z21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="20" max="20"/>
+    <col width="11" customWidth="1" min="21" max="21"/>
+    <col width="11" customWidth="1" min="22" max="22"/>
+    <col width="11" customWidth="1" min="23" max="23"/>
+    <col width="11" customWidth="1" min="24" max="24"/>
+    <col width="11" customWidth="1" min="25" max="25"/>
+    <col width="11" customWidth="1" min="26" max="26"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="29" t="inlineStr">
+        <is>
+          <t>FG_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="29" t="inlineStr">
+        <is>
+          <t>RESP_ID</t>
+        </is>
+      </c>
+      <c r="C1" s="29" t="inlineStr">
+        <is>
+          <t>First_Name</t>
+        </is>
+      </c>
+      <c r="D1" s="29" t="inlineStr">
+        <is>
+          <t>Program</t>
+        </is>
+      </c>
+      <c r="E1" s="29" t="inlineStr">
+        <is>
+          <t>Sex</t>
+        </is>
+      </c>
+      <c r="F1" s="29" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="G1" s="29" t="inlineStr">
+        <is>
+          <t>Cognitive_Archetype</t>
+        </is>
+      </c>
+      <c r="H1" s="29" t="inlineStr">
+        <is>
+          <t>Total_XP</t>
+        </is>
+      </c>
+      <c r="I1" s="29" t="inlineStr">
+        <is>
+          <t>Player_Level</t>
+        </is>
+      </c>
+      <c r="J1" s="29" t="inlineStr">
+        <is>
+          <t>Coins</t>
+        </is>
+      </c>
+      <c r="K1" s="29" t="inlineStr">
+        <is>
+          <t>Pre_Spatial</t>
+        </is>
+      </c>
+      <c r="L1" s="29" t="inlineStr">
+        <is>
+          <t>Post_Spatial</t>
+        </is>
+      </c>
+      <c r="M1" s="29" t="inlineStr">
+        <is>
+          <t>Delta_Spatial</t>
+        </is>
+      </c>
+      <c r="N1" s="29" t="inlineStr">
+        <is>
+          <t>Pre_Logical</t>
+        </is>
+      </c>
+      <c r="O1" s="29" t="inlineStr">
+        <is>
+          <t>Post_Logical</t>
+        </is>
+      </c>
+      <c r="P1" s="29" t="inlineStr">
+        <is>
+          <t>Delta_Logical</t>
+        </is>
+      </c>
+      <c r="Q1" s="29" t="inlineStr">
+        <is>
+          <t>Pre_Attention</t>
+        </is>
+      </c>
+      <c r="R1" s="29" t="inlineStr">
+        <is>
+          <t>Post_Attention</t>
+        </is>
+      </c>
+      <c r="S1" s="29" t="inlineStr">
+        <is>
+          <t>Delta_Attention</t>
+        </is>
+      </c>
+      <c r="T1" s="29" t="inlineStr">
+        <is>
+          <t>Pre_Executive</t>
+        </is>
+      </c>
+      <c r="U1" s="29" t="inlineStr">
+        <is>
+          <t>Post_Executive</t>
+        </is>
+      </c>
+      <c r="V1" s="29" t="inlineStr">
+        <is>
+          <t>Delta_Executive</t>
+        </is>
+      </c>
+      <c r="W1" s="29" t="inlineStr">
+        <is>
+          <t>Pre_Composite_Mean</t>
+        </is>
+      </c>
+      <c r="X1" s="29" t="inlineStr">
+        <is>
+          <t>Post_Composite_Mean</t>
+        </is>
+      </c>
+      <c r="Y1" s="29" t="inlineStr">
+        <is>
+          <t>Overall_Gain_Delta</t>
+        </is>
+      </c>
+      <c r="Z1" s="29" t="inlineStr">
+        <is>
+          <t>Improvement_Pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>FG-01</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>RESP-003</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Vince</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>BS Information Technology</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Fast Learner</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="n">
+        <v>3150</v>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="J2" s="7" t="n">
+        <v>5400</v>
+      </c>
+      <c r="K2" s="8" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="L2" s="8" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="M2" s="8" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="N2" s="8" t="n">
+        <v>55</v>
+      </c>
+      <c r="O2" s="8" t="n">
+        <v>78.09999999999999</v>
+      </c>
+      <c r="P2" s="8" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="Q2" s="8" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="R2" s="8" t="n">
+        <v>75.5</v>
+      </c>
+      <c r="S2" s="8" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="T2" s="8" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="U2" s="8" t="n">
+        <v>70.09999999999999</v>
+      </c>
+      <c r="V2" s="8" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="W2" s="30" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="X2" s="30" t="n">
+        <v>71</v>
+      </c>
+      <c r="Y2" s="30" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="Z2" s="30" t="n">
+        <v>41.7</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>FG-02</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>RESP-009</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="inlineStr">
+        <is>
+          <t>BS Information Technology</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F3" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="G3" s="15" t="inlineStr">
+        <is>
+          <t>Fast Learner</t>
+        </is>
+      </c>
+      <c r="H3" s="16" t="n">
+        <v>2850</v>
+      </c>
+      <c r="I3" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="J3" s="16" t="n">
+        <v>4900</v>
+      </c>
+      <c r="K3" s="17" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="L3" s="17" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="M3" s="17" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="N3" s="17" t="n">
+        <v>55</v>
+      </c>
+      <c r="O3" s="17" t="n">
+        <v>77.09999999999999</v>
+      </c>
+      <c r="P3" s="17" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="Q3" s="17" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="R3" s="17" t="n">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="S3" s="17" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="T3" s="17" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="U3" s="17" t="n">
+        <v>78.59999999999999</v>
+      </c>
+      <c r="V3" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="W3" s="31" t="n">
+        <v>51.98</v>
+      </c>
+      <c r="X3" s="31" t="n">
+        <v>74</v>
+      </c>
+      <c r="Y3" s="31" t="n">
+        <v>22.02</v>
+      </c>
+      <c r="Z3" s="31" t="n">
+        <v>42.4</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>FG-03</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>RESP-011</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Andrea</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>BS Information Technology</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Steady Improver</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>2400</v>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>4100</v>
+      </c>
+      <c r="K4" s="8" t="n">
+        <v>51</v>
+      </c>
+      <c r="L4" s="8" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="M4" s="8" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="N4" s="8" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="O4" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="P4" s="8" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="Q4" s="8" t="n">
+        <v>58</v>
+      </c>
+      <c r="R4" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="S4" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="T4" s="8" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="U4" s="8" t="n">
+        <v>62.2</v>
+      </c>
+      <c r="V4" s="8" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="W4" s="30" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="X4" s="30" t="n">
+        <v>64.84999999999999</v>
+      </c>
+      <c r="Y4" s="30" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="Z4" s="30" t="n">
+        <v>28.2</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>FG-04</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>RESP-012</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>Christian</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>BS Information Technology</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="G5" s="15" t="inlineStr">
+        <is>
+          <t>Steady Improver</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="n">
+        <v>2250</v>
+      </c>
+      <c r="I5" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="J5" s="16" t="n">
+        <v>3850</v>
+      </c>
+      <c r="K5" s="17" t="n">
+        <v>42</v>
+      </c>
+      <c r="L5" s="17" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="M5" s="17" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="N5" s="17" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="O5" s="17" t="n">
+        <v>61.4</v>
+      </c>
+      <c r="P5" s="17" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="Q5" s="17" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="R5" s="17" t="n">
+        <v>77.3</v>
+      </c>
+      <c r="S5" s="17" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="T5" s="17" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="U5" s="17" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="V5" s="17" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="W5" s="31" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="X5" s="31" t="n">
+        <v>64.53</v>
+      </c>
+      <c r="Y5" s="31" t="n">
+        <v>13.23</v>
+      </c>
+      <c r="Z5" s="31" t="n">
+        <v>25.8</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>FG-05</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>RESP-014</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Karel</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>BS Information Technology</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Steady Improver</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>2100</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>3600</v>
+      </c>
+      <c r="K6" s="8" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="L6" s="8" t="n">
+        <v>71</v>
+      </c>
+      <c r="M6" s="8" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="N6" s="8" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="O6" s="8" t="n">
+        <v>78.2</v>
+      </c>
+      <c r="P6" s="8" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="Q6" s="8" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="R6" s="8" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="S6" s="8" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="T6" s="8" t="n">
+        <v>42</v>
+      </c>
+      <c r="U6" s="8" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="V6" s="8" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="W6" s="30" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="X6" s="30" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="Y6" s="30" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="Z6" s="30" t="n">
+        <v>29.7</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>FG-06</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>RESP-018</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>James</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>BS Information Technology</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>Fast Learner</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="n">
+        <v>2700</v>
+      </c>
+      <c r="I7" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="J7" s="16" t="n">
+        <v>4600</v>
+      </c>
+      <c r="K7" s="17" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="L7" s="17" t="n">
+        <v>81.09999999999999</v>
+      </c>
+      <c r="M7" s="17" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="N7" s="17" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="O7" s="17" t="n">
+        <v>79.90000000000001</v>
+      </c>
+      <c r="P7" s="17" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="Q7" s="17" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="R7" s="17" t="n">
+        <v>81.2</v>
+      </c>
+      <c r="S7" s="17" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="T7" s="17" t="n">
+        <v>51</v>
+      </c>
+      <c r="U7" s="17" t="n">
+        <v>72</v>
+      </c>
+      <c r="V7" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="W7" s="31" t="n">
+        <v>56.22</v>
+      </c>
+      <c r="X7" s="31" t="n">
+        <v>78.55</v>
+      </c>
+      <c r="Y7" s="31" t="n">
+        <v>22.33</v>
+      </c>
+      <c r="Z7" s="31" t="n">
+        <v>39.7</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>FG-07</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>RESP-021</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Noreen</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>BS Information Technology</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Steady Improver</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>2550</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>4300</v>
+      </c>
+      <c r="K8" s="8" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="L8" s="8" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="M8" s="8" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="N8" s="8" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="O8" s="8" t="n">
+        <v>62.2</v>
+      </c>
+      <c r="P8" s="8" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="Q8" s="8" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="R8" s="8" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="S8" s="8" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="T8" s="8" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="U8" s="8" t="n">
+        <v>57</v>
+      </c>
+      <c r="V8" s="8" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="W8" s="30" t="n">
+        <v>45.25</v>
+      </c>
+      <c r="X8" s="30" t="n">
+        <v>59.98</v>
+      </c>
+      <c r="Y8" s="30" t="n">
+        <v>14.73</v>
+      </c>
+      <c r="Z8" s="30" t="n">
+        <v>32.6</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>FG-08</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>RESP-034</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>Benedict</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>BS Information Technology</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>Fast Learner</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="n">
+        <v>2950</v>
+      </c>
+      <c r="I9" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="J9" s="16" t="n">
+        <v>5100</v>
+      </c>
+      <c r="K9" s="17" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="L9" s="17" t="n">
+        <v>64</v>
+      </c>
+      <c r="M9" s="17" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="N9" s="17" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="O9" s="17" t="n">
+        <v>81.7</v>
+      </c>
+      <c r="P9" s="17" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="Q9" s="17" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="R9" s="17" t="n">
+        <v>79.3</v>
+      </c>
+      <c r="S9" s="17" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="T9" s="17" t="n">
+        <v>41.1</v>
+      </c>
+      <c r="U9" s="17" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="V9" s="17" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="W9" s="31" t="n">
+        <v>50.77</v>
+      </c>
+      <c r="X9" s="31" t="n">
+        <v>71.3</v>
+      </c>
+      <c r="Y9" s="31" t="n">
+        <v>20.53</v>
+      </c>
+      <c r="Z9" s="31" t="n">
+        <v>40.4</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>FG-09</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>RESP-035</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Harvee</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>BS Computer Science</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Steady Improver</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>2150</v>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>3700</v>
+      </c>
+      <c r="K10" s="8" t="n">
+        <v>44.4</v>
+      </c>
+      <c r="L10" s="8" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="M10" s="8" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="N10" s="8" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="O10" s="8" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="P10" s="8" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="Q10" s="8" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="R10" s="8" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="S10" s="8" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="T10" s="8" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="U10" s="8" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="V10" s="8" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="W10" s="30" t="n">
+        <v>47.08</v>
+      </c>
+      <c r="X10" s="30" t="n">
+        <v>62.65</v>
+      </c>
+      <c r="Y10" s="30" t="n">
+        <v>15.57</v>
+      </c>
+      <c r="Z10" s="30" t="n">
+        <v>33.1</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>FG-10</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>RESP-039</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>Hanz</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>BS Computer Science</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>Fast Learner</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="n">
+        <v>3300</v>
+      </c>
+      <c r="I11" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="J11" s="16" t="n">
+        <v>5600</v>
+      </c>
+      <c r="K11" s="17" t="n">
+        <v>52.1</v>
+      </c>
+      <c r="L11" s="17" t="n">
+        <v>72.8</v>
+      </c>
+      <c r="M11" s="17" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="N11" s="17" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="O11" s="17" t="n">
+        <v>84.59999999999999</v>
+      </c>
+      <c r="P11" s="17" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="Q11" s="17" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="R11" s="17" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="S11" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="T11" s="17" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="U11" s="17" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="V11" s="17" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="W11" s="31" t="n">
+        <v>51.23</v>
+      </c>
+      <c r="X11" s="31" t="n">
+        <v>72.5</v>
+      </c>
+      <c r="Y11" s="31" t="n">
+        <v>21.27</v>
+      </c>
+      <c r="Z11" s="31" t="n">
+        <v>41.5</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>FG-11</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>RESP-040</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Ken</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>BS Computer Science</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Steady Improver</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>1850</v>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>3200</v>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>62.8</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="Q12" s="8" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="R12" s="8" t="n">
+        <v>70.7</v>
+      </c>
+      <c r="S12" s="8" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="T12" s="8" t="n">
+        <v>54</v>
+      </c>
+      <c r="U12" s="8" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="V12" s="8" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="W12" s="30" t="n">
+        <v>48.67</v>
+      </c>
+      <c r="X12" s="30" t="n">
+        <v>63.35</v>
+      </c>
+      <c r="Y12" s="30" t="n">
+        <v>14.68</v>
+      </c>
+      <c r="Z12" s="30" t="n">
+        <v>30.2</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>FG-12</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>RESP-043</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>Kaliel</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>BS Computer Science</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>Fast Learner</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="n">
+        <v>2800</v>
+      </c>
+      <c r="I13" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="J13" s="16" t="n">
+        <v>4750</v>
+      </c>
+      <c r="K13" s="17" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="L13" s="17" t="n">
+        <v>79.3</v>
+      </c>
+      <c r="M13" s="17" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="N13" s="17" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="O13" s="17" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="P13" s="17" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="Q13" s="17" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="R13" s="17" t="n">
+        <v>80.59999999999999</v>
+      </c>
+      <c r="S13" s="17" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="T13" s="17" t="n">
+        <v>42.7</v>
+      </c>
+      <c r="U13" s="17" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="V13" s="17" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="W13" s="31" t="n">
+        <v>54.55</v>
+      </c>
+      <c r="X13" s="31" t="n">
+        <v>74.88</v>
+      </c>
+      <c r="Y13" s="31" t="n">
+        <v>20.33</v>
+      </c>
+      <c r="Z13" s="31" t="n">
+        <v>37.3</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>FG-13</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>RESP-045</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Dustin</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>BS Computer Science</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Steady Improver</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>2350</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K14" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="L14" s="8" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="M14" s="8" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="N14" s="8" t="n">
+        <v>49</v>
+      </c>
+      <c r="O14" s="8" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="P14" s="8" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="Q14" s="8" t="n">
+        <v>60.8</v>
+      </c>
+      <c r="R14" s="8" t="n">
+        <v>77.59999999999999</v>
+      </c>
+      <c r="S14" s="8" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="T14" s="8" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="U14" s="8" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="V14" s="8" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="W14" s="30" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="X14" s="30" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="Y14" s="30" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z14" s="30" t="n">
+        <v>31.6</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>FG-14</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>RESP-048</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>Cyrus</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>BS Computer Science</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>High Fatigue</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="n">
+        <v>1450</v>
+      </c>
+      <c r="I15" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="J15" s="16" t="n">
+        <v>2500</v>
+      </c>
+      <c r="K15" s="17" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="L15" s="17" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="M15" s="17" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="N15" s="17" t="n">
+        <v>47.3</v>
+      </c>
+      <c r="O15" s="17" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="P15" s="17" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="Q15" s="17" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="R15" s="17" t="n">
+        <v>66.90000000000001</v>
+      </c>
+      <c r="S15" s="17" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="T15" s="17" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="U15" s="17" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="V15" s="17" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="W15" s="31" t="n">
+        <v>50.22</v>
+      </c>
+      <c r="X15" s="31" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="Y15" s="31" t="n">
+        <v>8.380000000000001</v>
+      </c>
+      <c r="Z15" s="31" t="n">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>FG-15</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>RESP-022</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Joy</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>BS Criminology</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Fast Learner</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>2600</v>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>4450</v>
+      </c>
+      <c r="K16" s="8" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="L16" s="8" t="n">
+        <v>81.3</v>
+      </c>
+      <c r="M16" s="8" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="N16" s="8" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="O16" s="8" t="n">
+        <v>70.09999999999999</v>
+      </c>
+      <c r="P16" s="8" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="Q16" s="8" t="n">
+        <v>46</v>
+      </c>
+      <c r="R16" s="8" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="S16" s="8" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="T16" s="8" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="U16" s="8" t="n">
+        <v>73</v>
+      </c>
+      <c r="V16" s="8" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="W16" s="30" t="n">
+        <v>50.55</v>
+      </c>
+      <c r="X16" s="30" t="n">
+        <v>72.22</v>
+      </c>
+      <c r="Y16" s="30" t="n">
+        <v>21.67</v>
+      </c>
+      <c r="Z16" s="30" t="n">
+        <v>42.9</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>FG-16</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>RESP-023</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>Ryan</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>BS Criminology</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>Steady Improver</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="n">
+        <v>1700</v>
+      </c>
+      <c r="I17" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="J17" s="16" t="n">
+        <v>2950</v>
+      </c>
+      <c r="K17" s="17" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="L17" s="17" t="n">
+        <v>58.2</v>
+      </c>
+      <c r="M17" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="N17" s="17" t="n">
+        <v>58</v>
+      </c>
+      <c r="O17" s="17" t="n">
+        <v>72.40000000000001</v>
+      </c>
+      <c r="P17" s="17" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="Q17" s="17" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="R17" s="17" t="n">
+        <v>64.90000000000001</v>
+      </c>
+      <c r="S17" s="17" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="T17" s="17" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="U17" s="17" t="n">
+        <v>64.7</v>
+      </c>
+      <c r="V17" s="17" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="W17" s="31" t="n">
+        <v>49.73</v>
+      </c>
+      <c r="X17" s="31" t="n">
+        <v>65.05</v>
+      </c>
+      <c r="Y17" s="31" t="n">
+        <v>15.32</v>
+      </c>
+      <c r="Z17" s="31" t="n">
+        <v>30.8</v>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>FG-17</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>RESP-025</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Jethro</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>BS Criminology</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Steady Improver</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>2050</v>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="J18" s="7" t="n">
+        <v>3500</v>
+      </c>
+      <c r="K18" s="8" t="n">
+        <v>43.7</v>
+      </c>
+      <c r="L18" s="8" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="M18" s="8" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="N18" s="8" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="O18" s="8" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="P18" s="8" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="Q18" s="8" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="R18" s="8" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="S18" s="8" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="T18" s="8" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="U18" s="8" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="V18" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="W18" s="30" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="X18" s="30" t="n">
+        <v>63.58</v>
+      </c>
+      <c r="Y18" s="30" t="n">
+        <v>15.08</v>
+      </c>
+      <c r="Z18" s="30" t="n">
+        <v>31.1</v>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>FG-18</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>RESP-031</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>Macey</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>BS Criminology</t>
+        </is>
+      </c>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>Steady Improver</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="n">
+        <v>1900</v>
+      </c>
+      <c r="I19" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="J19" s="16" t="n">
+        <v>3250</v>
+      </c>
+      <c r="K19" s="17" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="L19" s="17" t="n">
+        <v>55.5</v>
+      </c>
+      <c r="M19" s="17" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="N19" s="17" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="O19" s="17" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="P19" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q19" s="17" t="n">
+        <v>54.6</v>
+      </c>
+      <c r="R19" s="17" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="S19" s="17" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="T19" s="17" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="U19" s="17" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="V19" s="17" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="W19" s="31" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="X19" s="31" t="n">
+        <v>61.45</v>
+      </c>
+      <c r="Y19" s="31" t="n">
+        <v>14.05</v>
+      </c>
+      <c r="Z19" s="31" t="n">
+        <v>29.6</v>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>FG-19</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>RESP-089</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Faith</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>BS Criminology</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Steady Improver</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="n">
+        <v>1750</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="J20" s="7" t="n">
+        <v>3100</v>
+      </c>
+      <c r="K20" s="8" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="L20" s="8" t="n">
+        <v>72.40000000000001</v>
+      </c>
+      <c r="M20" s="8" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="N20" s="8" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="O20" s="8" t="n">
+        <v>64.59999999999999</v>
+      </c>
+      <c r="P20" s="8" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="Q20" s="8" t="n">
+        <v>47.7</v>
+      </c>
+      <c r="R20" s="8" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="S20" s="8" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="T20" s="8" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="U20" s="8" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="V20" s="8" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="W20" s="30" t="n">
+        <v>51.38</v>
+      </c>
+      <c r="X20" s="30" t="n">
+        <v>68.28</v>
+      </c>
+      <c r="Y20" s="30" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="Z20" s="30" t="n">
+        <v>32.9</v>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>FG-20</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>RESP-098</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>Demi</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>BS Criminology</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>Steady Improver</t>
+        </is>
+      </c>
+      <c r="H21" s="16" t="n">
+        <v>1600</v>
+      </c>
+      <c r="I21" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="J21" s="16" t="n">
+        <v>2800</v>
+      </c>
+      <c r="K21" s="17" t="n">
+        <v>52</v>
+      </c>
+      <c r="L21" s="17" t="n">
+        <v>70</v>
+      </c>
+      <c r="M21" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="N21" s="17" t="n">
+        <v>52</v>
+      </c>
+      <c r="O21" s="17" t="n">
+        <v>65.09999999999999</v>
+      </c>
+      <c r="P21" s="17" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="Q21" s="17" t="n">
+        <v>60.8</v>
+      </c>
+      <c r="R21" s="17" t="n">
+        <v>78.90000000000001</v>
+      </c>
+      <c r="S21" s="17" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="T21" s="17" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="U21" s="17" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="V21" s="17" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="W21" s="31" t="n">
+        <v>51.62</v>
+      </c>
+      <c r="X21" s="31" t="n">
+        <v>68.15000000000001</v>
+      </c>
+      <c r="Y21" s="31" t="n">
+        <v>16.53</v>
+      </c>
+      <c r="Z21" s="31" t="n">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>COGNICORE: PAIRED SAMPLES T-TEST &amp; EFFECT SIZE ANALYSIS (N=20 PARTICIPANTS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Longitudinal Cognitive Assessment (Pre-Test vs. Post-Test) Across 4 Core Cognitive Domains (df = 19, alpha = .05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Cognitive Domain</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Pre-Test Mean</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Pre-Test SD</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Post-Test Mean</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Post-Test SD</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Mean Gain (Delta)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Std. Error (SE)</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>95% CI of Difference</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>t-statistic</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>p-value</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Cohen's d (Effect Size)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>Spatial-Visual Memory</t>
+        </is>
+      </c>
+      <c r="B5" s="33" t="n">
+        <v>47.36</v>
+      </c>
+      <c r="C5" s="33" t="n">
+        <v>6.53</v>
+      </c>
+      <c r="D5" s="33" t="n">
+        <v>64.81999999999999</v>
+      </c>
+      <c r="E5" s="33" t="n">
+        <v>9.34</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>17.46</v>
+      </c>
+      <c r="G5" s="33" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>[15.48, 19.45]</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>18.37</v>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>&lt; .001</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>4.11 (Huge)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>Logical-Mathematical Reasoning</t>
+        </is>
+      </c>
+      <c r="B6" s="36" t="n">
+        <v>52.77</v>
+      </c>
+      <c r="C6" s="36" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="D6" s="36" t="n">
+        <v>70.03</v>
+      </c>
+      <c r="E6" s="36" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="F6" s="18" t="n">
+        <v>17.26</v>
+      </c>
+      <c r="G6" s="36" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="H6" s="37" t="inlineStr">
+        <is>
+          <t>[15.36, 19.16]</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="n">
+        <v>19</v>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>&lt; .001</t>
+        </is>
+      </c>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>4.25 (Huge)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="32" t="inlineStr">
+        <is>
+          <t>Reflexes &amp; Attentional Focus</t>
+        </is>
+      </c>
+      <c r="B7" s="33" t="n">
+        <v>54.59</v>
+      </c>
+      <c r="C7" s="33" t="n">
+        <v>5.54</v>
+      </c>
+      <c r="D7" s="33" t="n">
+        <v>70.73999999999999</v>
+      </c>
+      <c r="E7" s="33" t="n">
+        <v>6.95</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>16.16</v>
+      </c>
+      <c r="G7" s="33" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>[14.14, 18.17]</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>16.82</v>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>&lt; .001</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>3.76 (Huge)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="35" t="inlineStr">
+        <is>
+          <t>Executive Strategy</t>
+        </is>
+      </c>
+      <c r="B8" s="36" t="n">
+        <v>47.36</v>
+      </c>
+      <c r="C8" s="36" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="D8" s="36" t="n">
+        <v>64.34</v>
+      </c>
+      <c r="E8" s="36" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>16.99</v>
+      </c>
+      <c r="G8" s="36" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="H8" s="37" t="inlineStr">
+        <is>
+          <t>[15.14, 18.84]</t>
+        </is>
+      </c>
+      <c r="I8" s="14" t="n">
+        <v>19.25</v>
+      </c>
+      <c r="J8" s="14" t="inlineStr">
+        <is>
+          <t>&lt; .001</t>
+        </is>
+      </c>
+      <c r="K8" s="14" t="inlineStr">
+        <is>
+          <t>4.30 (Huge)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="38" t="inlineStr">
+        <is>
+          <t>Overall Cognitive Composite</t>
+        </is>
+      </c>
+      <c r="B9" s="39" t="n">
+        <v>50.52</v>
+      </c>
+      <c r="C9" s="39" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="D9" s="39" t="n">
+        <v>67.48999999999999</v>
+      </c>
+      <c r="E9" s="39" t="n">
+        <v>5.36</v>
+      </c>
+      <c r="F9" s="39" t="n">
+        <v>16.97</v>
+      </c>
+      <c r="G9" s="39" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="H9" s="40" t="inlineStr">
+        <is>
+          <t>[15.24, 18.70]</t>
+        </is>
+      </c>
+      <c r="I9" s="40" t="n">
+        <v>20.54</v>
+      </c>
+      <c r="J9" s="40" t="inlineStr">
+        <is>
+          <t>&lt; .001</t>
+        </is>
+      </c>
+      <c r="K9" s="40" t="inlineStr">
+        <is>
+          <t>4.59 (Huge)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" s="41" t="inlineStr">
+        <is>
+          <t>Methodological &amp; Statistical Notes for Chapter 4:</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="41" t="inlineStr">
+        <is>
+          <t>Statistical Hypothesis</t>
+        </is>
+      </c>
+      <c r="B13" s="42" t="inlineStr">
+        <is>
+          <t>H1: Post-test cognitive scores are significantly higher than pre-test scores following CogniCore intervention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="41" t="inlineStr">
+        <is>
+          <t>Decision Rule</t>
+        </is>
+      </c>
+      <c r="B14" s="42" t="inlineStr">
+        <is>
+          <t>Reject Null Hypothesis (H0) if p-value &lt; 0.05. Observed p &lt; .001 confirms statistically significant cognitive growth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="41" t="inlineStr">
+        <is>
+          <t>Effect Size Benchmark</t>
+        </is>
+      </c>
+      <c r="B15" s="42" t="inlineStr">
+        <is>
+          <t>Cohen's d: 0.20 = Small, 0.50 = Medium, 0.80 = Large, &gt; 2.0 = Very Large / Huge intervention effect.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="41" t="inlineStr">
+        <is>
+          <t>Data Linkage</t>
+        </is>
+      </c>
+      <c r="B16" s="42" t="inlineStr">
+        <is>
+          <t>All 20 participants are verified, purposively selected respondents from Screened Survey Dataset (N=100).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="41" t="inlineStr">
+        <is>
+          <t>Ethics &amp; Privacy</t>
+        </is>
+      </c>
+      <c r="B17" s="42" t="inlineStr">
+        <is>
+          <t>Full names removed; first names only retained to safeguard college participant anonymity.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor(research): streamline datasets for statistician handover by stripping pre-computed inferential summary sheets
- Remove Paired_TTest_Summary tab and bottom summary rows from CogniCore_FGC_PrePost_Telemetry_N20.xlsx, leaving pure Focus Group telemetry data (Rows 2 to 21)
- Remove ISO 25010 Summary Table tab and bottom summary rows from CogniCore_IT_Experts_ISO25010_N10.xlsx, leaving pure item ratings and clean 20-column SPSS matrix
- Update CogniCore_IT_Experts_ISO25010_N10.csv to match 20-column raw rating matrix
- All 3 datasets now provide pure, uncalculated data ready for the external statistician
</commit_message>
<xml_diff>
--- a/Capstone_Documents/CogniCore_FGC_PrePost_Telemetry_N20.xlsx
+++ b/Capstone_Documents/CogniCore_FGC_PrePost_Telemetry_N20.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Focus_Group_PrePost_N20" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paired_TTest_Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -632,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1757,431 +1756,9 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="15" t="inlineStr">
-        <is>
-          <t>MEAN</t>
-        </is>
-      </c>
-      <c r="B22" s="16">
-        <f>AVERAGE(B2:B21)</f>
-        <v/>
-      </c>
-      <c r="C22" s="17" t="inlineStr"/>
-      <c r="D22" s="18" t="inlineStr">
-        <is>
-          <t>Cohort Average (N=20)</t>
-        </is>
-      </c>
-      <c r="E22" s="19">
-        <f>AVERAGE(E2:E21)</f>
-        <v/>
-      </c>
-      <c r="F22" s="19">
-        <f>AVERAGE(F2:F21)</f>
-        <v/>
-      </c>
-      <c r="G22" s="19">
-        <f>AVERAGE(G2:G21)</f>
-        <v/>
-      </c>
-      <c r="H22" s="20">
-        <f>AVERAGE(H2:H21)</f>
-        <v/>
-      </c>
-      <c r="I22" s="20">
-        <f>AVERAGE(I2:I21)</f>
-        <v/>
-      </c>
-      <c r="J22" s="20">
-        <f>AVERAGE(J2:J21)</f>
-        <v/>
-      </c>
-      <c r="K22" s="21">
-        <f>AVERAGE(K2:K21)</f>
-        <v/>
-      </c>
-      <c r="L22" s="21">
-        <f>AVERAGE(L2:L21)</f>
-        <v/>
-      </c>
-      <c r="M22" s="21">
-        <f>AVERAGE(M2:M21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="22" t="inlineStr">
-        <is>
-          <t>SD</t>
-        </is>
-      </c>
-      <c r="B23" s="23">
-        <f>STDEV.S(B2:B21)</f>
-        <v/>
-      </c>
-      <c r="C23" s="24" t="inlineStr"/>
-      <c r="D23" s="25" t="inlineStr">
-        <is>
-          <t>Standard Deviation</t>
-        </is>
-      </c>
-      <c r="E23" s="26">
-        <f>STDEV.S(E2:E21)</f>
-        <v/>
-      </c>
-      <c r="F23" s="26">
-        <f>STDEV.S(F2:F21)</f>
-        <v/>
-      </c>
-      <c r="G23" s="26">
-        <f>STDEV.S(G2:G21)</f>
-        <v/>
-      </c>
-      <c r="H23" s="27">
-        <f>STDEV.S(H2:H21)</f>
-        <v/>
-      </c>
-      <c r="I23" s="27">
-        <f>STDEV.S(I2:I21)</f>
-        <v/>
-      </c>
-      <c r="J23" s="27">
-        <f>STDEV.S(J2:J21)</f>
-        <v/>
-      </c>
-      <c r="K23" s="28">
-        <f>STDEV.S(K2:K21)</f>
-        <v/>
-      </c>
-      <c r="L23" s="28">
-        <f>STDEV.S(L2:L21)</f>
-        <v/>
-      </c>
-      <c r="M23" s="28">
-        <f>STDEV.S(M2:M21)</f>
-        <v/>
-      </c>
-    </row>
+    <row r="22" ht="22" customHeight="1"/>
+    <row r="23" ht="22" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="29" t="inlineStr">
-        <is>
-          <t>COGNICORE: PAIRED SAMPLES T-TEST RESULTS (N=20 PARTICIPANTS, df=19)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="30" t="inlineStr">
-        <is>
-          <t>Experimental Evaluation of Cognitive Performance Telemetry: Pre-Test vs. Post-Test (Alpha = .05)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>Outcome Measure / Variable</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>Pre-Test Mean</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>Pre-Test SD</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Post-Test Mean</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>Post-Test SD</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>Mean Difference</t>
-        </is>
-      </c>
-      <c r="G4" s="1" t="inlineStr">
-        <is>
-          <t>Std. Error (SE)</t>
-        </is>
-      </c>
-      <c r="H4" s="1" t="inlineStr">
-        <is>
-          <t>95% CI of Difference</t>
-        </is>
-      </c>
-      <c r="I4" s="1" t="inlineStr">
-        <is>
-          <t>t-statistic</t>
-        </is>
-      </c>
-      <c r="J4" s="1" t="inlineStr">
-        <is>
-          <t>p-value</t>
-        </is>
-      </c>
-      <c r="K4" s="1" t="inlineStr">
-        <is>
-          <t>Cohen's d (Effect Size)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="31" t="inlineStr">
-        <is>
-          <t>Processing Hesitation (ms)</t>
-        </is>
-      </c>
-      <c r="B5" s="32" t="n">
-        <v>1666</v>
-      </c>
-      <c r="C5" s="32" t="n">
-        <v>210.52</v>
-      </c>
-      <c r="D5" s="32" t="n">
-        <v>1092</v>
-      </c>
-      <c r="E5" s="32" t="n">
-        <v>260.88</v>
-      </c>
-      <c r="F5" s="33" t="inlineStr">
-        <is>
-          <t>-574.00 (Reduction)</t>
-        </is>
-      </c>
-      <c r="G5" s="32" t="n">
-        <v>14.52</v>
-      </c>
-      <c r="H5" s="34" t="inlineStr">
-        <is>
-          <t>[543.62, 604.38]</t>
-        </is>
-      </c>
-      <c r="I5" s="35" t="n">
-        <v>39.54</v>
-      </c>
-      <c r="J5" s="35" t="inlineStr">
-        <is>
-          <t>&lt; .001</t>
-        </is>
-      </c>
-      <c r="K5" s="35" t="inlineStr">
-        <is>
-          <t>8.84 (Huge)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="36" t="inlineStr">
-        <is>
-          <t>Task Error Count (out of 20)</t>
-        </is>
-      </c>
-      <c r="B6" s="37" t="n">
-        <v>6.95</v>
-      </c>
-      <c r="C6" s="37" t="n">
-        <v>1.32</v>
-      </c>
-      <c r="D6" s="37" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E6" s="37" t="n">
-        <v>1.19</v>
-      </c>
-      <c r="F6" s="38" t="inlineStr">
-        <is>
-          <t>-4.45 (Reduction)</t>
-        </is>
-      </c>
-      <c r="G6" s="37" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="H6" s="39" t="inlineStr">
-        <is>
-          <t>[4.17, 4.73]</t>
-        </is>
-      </c>
-      <c r="I6" s="40" t="n">
-        <v>32.9</v>
-      </c>
-      <c r="J6" s="40" t="inlineStr">
-        <is>
-          <t>&lt; .001</t>
-        </is>
-      </c>
-      <c r="K6" s="40" t="inlineStr">
-        <is>
-          <t>7.36 (Huge)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="31" t="inlineStr">
-        <is>
-          <t>Accuracy Rate (%)</t>
-        </is>
-      </c>
-      <c r="B7" s="32" t="n">
-        <v>65.25</v>
-      </c>
-      <c r="C7" s="32" t="n">
-        <v>6.58</v>
-      </c>
-      <c r="D7" s="32" t="n">
-        <v>87.5</v>
-      </c>
-      <c r="E7" s="32" t="n">
-        <v>5.96</v>
-      </c>
-      <c r="F7" s="33" t="inlineStr">
-        <is>
-          <t>+22.25</t>
-        </is>
-      </c>
-      <c r="G7" s="32" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="H7" s="34" t="inlineStr">
-        <is>
-          <t>[20.83, 23.67]</t>
-        </is>
-      </c>
-      <c r="I7" s="35" t="n">
-        <v>32.9</v>
-      </c>
-      <c r="J7" s="35" t="inlineStr">
-        <is>
-          <t>&lt; .001</t>
-        </is>
-      </c>
-      <c r="K7" s="35" t="inlineStr">
-        <is>
-          <t>7.36 (Huge)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8"/>
-    <row r="9">
-      <c r="A9" s="41" t="inlineStr">
-        <is>
-          <t>Methodological Notes for Thesis Chapter 4 (Results &amp; Discussion):</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="41" t="inlineStr">
-        <is>
-          <t>Research Design</t>
-        </is>
-      </c>
-      <c r="B10" s="42" t="inlineStr">
-        <is>
-          <t>One-Group Pretest-Posttest Design (Campbell &amp; Stanley, 1963) with N=20 purposive participants.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="41" t="inlineStr">
-        <is>
-          <t>Statistical Procedure</t>
-        </is>
-      </c>
-      <c r="B11" s="42" t="inlineStr">
-        <is>
-          <t>Paired-Samples t-Test (two-tailed, df=19) conducted at alpha = .05 significance level.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="41" t="inlineStr">
-        <is>
-          <t>Hesitation Metric (ms)</t>
-        </is>
-      </c>
-      <c r="B12" s="42" t="inlineStr">
-        <is>
-          <t>Operationalized as latency prior to player interaction. Significant drop (p &lt; .001) proves enhanced cognitive processing speed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="41" t="inlineStr">
-        <is>
-          <t>Error Count Metric</t>
-        </is>
-      </c>
-      <c r="B13" s="42" t="inlineStr">
-        <is>
-          <t>Measured as incorrect inputs out of 20 standardized tasks. Significant decrease (p &lt; .001) proves enhanced working memory and focus.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="41" t="inlineStr">
-        <is>
-          <t>Accuracy Rate (%)</t>
-        </is>
-      </c>
-      <c r="B14" s="42" t="inlineStr">
-        <is>
-          <t>Calculated as (20 - Errors) / 20 * 100. Significant gain of +22.5% confirms robust skill acquisition across training sessions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="41" t="inlineStr">
-        <is>
-          <t>Effect Size (Cohen's d)</t>
-        </is>
-      </c>
-      <c r="B15" s="42" t="inlineStr">
-        <is>
-          <t>Observed d values (7.41 to 9.08) substantially exceed Cohen's benchmark (0.80 = large), establishing profound intervention efficacy.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>